<commit_message>
changing main.py to reduce logging information for the function app to svae costs
</commit_message>
<xml_diff>
--- a/backend/assets/data/fujitsu_capacities_calculated.xlsx
+++ b/backend/assets/data/fujitsu_capacities_calculated.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pardigmpartners-my.sharepoint.com/personal/alex_paradigm-esco_com/Documents/data_operations/ashp_calculator/backend/assets/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="323" documentId="13_ncr:1_{D420F103-AC1D-4B35-A441-D57FBF080E0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2ADA4DA6-6CDF-4987-9DFE-B82EF0220CBB}"/>
+  <xr:revisionPtr revIDLastSave="343" documentId="13_ncr:1_{D420F103-AC1D-4B35-A441-D57FBF080E0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0DFA0FDB-8579-4C8C-83E3-AA788D948DA4}"/>
   <bookViews>
-    <workbookView xWindow="48710" yWindow="260" windowWidth="27700" windowHeight="17110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="1680" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="indoor_combinations" sheetId="2" r:id="rId1"/>
     <sheet name="capacity_70_0" sheetId="1" r:id="rId2"/>
+    <sheet name="unique_models" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -34,6 +35,28 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -20299,4 +20322,90 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39B9EFDB-256D-455A-A628-9BDA09879C73}">
+  <dimension ref="A1:A15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" t="str" cm="1">
+        <f t="array" ref="A1:A15">_xlfn.UNIQUE(indoor_combinations!A:A)</f>
+        <v>Model</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2" t="str">
+        <v>AOUH18KWAH2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" t="str">
+        <v>AOUH24KWAH3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4" t="str">
+        <v>AOUH36KWAH4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A5" t="str">
+        <v>AOUH12KUAS1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A6" t="str">
+        <v>AOUH18KUAS1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A7" t="str">
+        <v>AOUH24KUAS1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A8" t="str">
+        <v>AOUH30KUAS1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A9" t="str">
+        <v>AOUH36KUAS1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A10" t="str">
+        <v>AOUH48KUAS1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A11" t="str">
+        <v>AOUH30KUAH1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A12" t="str">
+        <v>AOUH36KUAH1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A13" t="str">
+        <v>AOUH48KUAH1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A14" t="str">
+        <v>AOUH45KWAS5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>